<commit_message>
Update Excel files and modify date formats in scripts
- Updated multiple Excel files in the MONOPUNTO and MULTIPUNTO directories, reflecting changes in data.
- Adjusted date formats in the `llenar_planillas.py` script to 'DD/MM/YYYY' for 'Recibida', 'Vencimiento', and 'Validez' columns.
- Changed date pattern in `procesar_ofertas.py` for DateEntry widgets to 'dd/mm/yyyy' for consistency in date handling.
</commit_message>
<xml_diff>
--- a/MONOPUNTO/212 Datos Monopunto RECTYAFIL.xlsx
+++ b/MONOPUNTO/212 Datos Monopunto RECTYAFIL.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,7 +51,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,6 +419,22 @@
   </sheetPr>
   <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -498,13 +515,13 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="C2" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="D2" s="1" t="n">
         <v>46568</v>
-      </c>
-      <c r="D2" s="1" t="n">
-        <v>46199</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -548,13 +565,13 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="C3" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>46568</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>46199</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -598,13 +615,13 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="C4" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="D4" s="1" t="n">
         <v>46568</v>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>46199</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -648,13 +665,13 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="C5" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="D5" s="1" t="n">
         <v>46568</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>46199</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update multiple Excel files and enhance the 'llenar_planillas.py' script
- Modified various Excel files in the MONOPUNTO and MULTIPUNTO directories, indicating binary differences.
- Enhanced the 'llenar_planillas.py' script to improve client code handling and file naming conventions:
  - Introduced an effective key for clients based on existing codes.
  - Updated the logic for generating file names to include the primary code.
  - Added validation to ensure the correct client codes match the file names.
</commit_message>
<xml_diff>
--- a/MONOPUNTO/212 Datos Monopunto RECTYAFIL.xlsx
+++ b/MONOPUNTO/212 Datos Monopunto RECTYAFIL.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +48,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +423,7 @@
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -514,15 +514,11 @@
           <t>ELEIA</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="D2" s="1" t="n">
-        <v>46568</v>
-      </c>
+      <c r="B2" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>No</t>
@@ -564,15 +560,11 @@
           <t>ELEIA</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>46568</v>
-      </c>
+      <c r="B3" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>No</t>
@@ -614,15 +606,11 @@
           <t>IBERDROLA</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>46568</v>
-      </c>
+      <c r="B4" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>No</t>
@@ -664,15 +652,11 @@
           <t>IBERDROLA</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>46197</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>46568</v>
-      </c>
+      <c r="B5" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>No</t>

</xml_diff>